<commit_message>
Fixed order for the legends
</commit_message>
<xml_diff>
--- a/20240325_Er/output/20240325_Er_element_pairs.xlsx
+++ b/20240325_Er/output/20240325_Er_element_pairs.xlsx
@@ -8,10 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Er-Co" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Er-In" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="In-In" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Co-Co" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Co-In" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="In-In" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Er-In" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -502,11 +500,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3.055</v>
+        <v>3.009</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>full_occupancy_atomic_mixing</t>
+          <t>full_occupancy</t>
         </is>
       </c>
     </row>
@@ -548,103 +546,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3.009</v>
+        <v>3.004</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>full_occupancy</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>File</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Distance</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Atomic Mixing</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1814810.cif</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>2.964</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>deficiency</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>File</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Distance</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Atomic Mixing</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1814810.cif</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>2.964</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>deficiency</t>
+          <t>full_occupancy_atomic_mixing</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add bin width per sheet
</commit_message>
<xml_diff>
--- a/20240325_Er/output/20240325_Er_element_pairs.xlsx
+++ b/20240325_Er/output/20240325_Er_element_pairs.xlsx
@@ -7,11 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Co-In" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Er-In" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Er-Co" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Co-Co" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Er-In" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="In-In" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="In-In" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -456,11 +454,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.964</v>
+        <v>3.004</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>deficiency</t>
+          <t>full_occupancy_atomic_mixing</t>
         </is>
       </c>
     </row>
@@ -548,98 +546,6 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.964</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>deficiency</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>File</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Distance</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Atomic Mixing</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1814810.cif</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>3.055</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>full_occupancy_atomic_mixing</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>File</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Distance</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Atomic Mixing</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1814810.cif</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
         <v>3.009</v>
       </c>
       <c r="C2" t="inlineStr">

</xml_diff>

<commit_message>
Add std and avg for excel
</commit_message>
<xml_diff>
--- a/20240325_Er/output/20240325_Er_element_pairs.xlsx
+++ b/20240325_Er/output/20240325_Er_element_pairs.xlsx
@@ -7,9 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Er-In" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Er-Co" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="In-In" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Er-Co" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="In-In" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Er-In" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Co-In" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Co-Co" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,13 +456,38 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3.004</v>
+        <v>2.623</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>full_occupancy_atomic_mixing</t>
-        </is>
-      </c>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2.623</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -473,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -500,13 +527,38 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.623</v>
+        <v>3.009</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>full_occupancy</t>
-        </is>
-      </c>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3.009</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -519,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -546,13 +598,180 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3.009</v>
+        <v>3.055</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>full_occupancy</t>
-        </is>
-      </c>
+          <t>Full occupancy with atomic mixing</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3.055</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Atomic Mixing</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1814810.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2.964</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Deficiency with atomic mixing</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2.964</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Atomic Mixing</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1814810.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2.964</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Deficiency with atomic mixing</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2.964</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>